<commit_message>
feat: add AttendanceSeeder and dataset for 15 employee trial logs
</commit_message>
<xml_diff>
--- a/database/seeders/Data_Absensi_15_Karyawan.xlsx
+++ b/database/seeders/Data_Absensi_15_Karyawan.xlsx
@@ -1896,19 +1896,19 @@
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>94.29000000000001</v>
+        <v>68.45</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0.0457</v>
+        <v>0.5821</v>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Cocok (Diterima)</t>
+          <t>Tidak Cocok (Ditolak)</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>DISETUJUI (Tepat Waktu)</t>
+          <t>GAGAL (Wajah Tidak Cocok)</t>
         </is>
       </c>
     </row>
@@ -3271,19 +3271,19 @@
         </is>
       </c>
       <c r="J51" s="2" t="n">
-        <v>10.37</v>
+        <v>82.75</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0.717</v>
+        <v>0.5185</v>
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>Tidak Cocok (Ditolak)</t>
+          <t>Cocok (Diterima)</t>
         </is>
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>GAGAL (Wajah Tidak Cocok)</t>
+          <t>DISETUJUI (Tepat Waktu)</t>
         </is>
       </c>
     </row>
@@ -3546,19 +3546,19 @@
         </is>
       </c>
       <c r="J56" s="2" t="n">
-        <v>90.63</v>
+        <v>71.20</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0.075</v>
+        <v>0.5644</v>
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>Cocok (Diterima)</t>
+          <t>Tidak Cocok (Ditolak)</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>DISETUJUI (Tepat Waktu)</t>
+          <t>GAGAL (Wajah Tidak Cocok)</t>
         </is>
       </c>
     </row>
@@ -5196,19 +5196,19 @@
         </is>
       </c>
       <c r="J86" s="2" t="n">
-        <v>88.47</v>
+        <v>66.80</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0.0922</v>
+        <v>0.5912</v>
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>Cocok (Diterima)</t>
+          <t>Tidak Cocok (Ditolak)</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>DISETUJUI (Tepat Waktu)</t>
+          <t>GAGAL (Wajah Tidak Cocok)</t>
         </is>
       </c>
     </row>
@@ -6571,19 +6571,19 @@
         </is>
       </c>
       <c r="J111" s="2" t="n">
-        <v>19.42</v>
+        <v>84.10</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>0.6446</v>
+        <v>0.4950</v>
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>Tidak Cocok (Ditolak)</t>
+          <t>Cocok (Diterima)</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr">
         <is>
-          <t>GAGAL (Wajah Tidak Cocok)</t>
+          <t>DISETUJUI (Tepat Waktu)</t>
         </is>
       </c>
     </row>
@@ -6846,19 +6846,19 @@
         </is>
       </c>
       <c r="J116" s="2" t="n">
-        <v>98.26000000000001</v>
+        <v>69.50</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>0.0139</v>
+        <v>0.5750</v>
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>Cocok (Diterima)</t>
+          <t>Tidak Cocok (Ditolak)</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr">
         <is>
-          <t>DISETUJUI (Tepat Waktu)</t>
+          <t>GAGAL (Wajah Tidak Cocok)</t>
         </is>
       </c>
     </row>
@@ -8496,19 +8496,19 @@
         </is>
       </c>
       <c r="J146" s="2" t="n">
-        <v>91.3</v>
+        <v>67.15</v>
       </c>
       <c r="K146" s="2" t="n">
-        <v>0.0696</v>
+        <v>0.5890</v>
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>Cocok (Diterima)</t>
+          <t>Tidak Cocok (Ditolak)</t>
         </is>
       </c>
       <c r="M146" s="3" t="inlineStr">
         <is>
-          <t>DISETUJUI (Tepat Waktu)</t>
+          <t>GAGAL (Wajah Tidak Cocok)</t>
         </is>
       </c>
     </row>

</xml_diff>